<commit_message>
Add inference results and update statistics outputs
Added new inference result files for group 609 across multiple dates and categories. Updated accuracy reports and added new accuracy result files for groups 90, 100, and 609. Modified numerous statistical output and result files for all groups, reflecting updated or new analysis results.
</commit_message>
<xml_diff>
--- a/inference_acc.xlsx
+++ b/inference_acc.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G15"/>
+  <dimension ref="A1:G21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -954,6 +954,216 @@
       <c r="G15" t="inlineStr">
         <is>
           <t>0.0018/ 40</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>21646</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>0.8636/ 18694</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>0.0721/ 1560</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>0.02/ 434</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>0.0163/ 352</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>0.0261/ 566</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>0.0018/ 40</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>21646</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>0.5383/ 11651</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>0.1655/ 3582</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>0.0667/ 1443</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>0.0966/ 2092</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>0.0931/ 2016</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>0.0398/ 862</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>21646</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>0.8636/ 18694</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>0.0721/ 1560</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>0.02/ 434</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>0.0163/ 352</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>0.0261/ 566</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>0.0018/ 40</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>21646</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>0.5383/ 11651</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>0.1655/ 3582</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>0.0667/ 1443</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>0.0966/ 2092</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>0.0931/ 2016</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>0.0398/ 862</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>21646</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>0.5315/ 11504</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>0.1702/ 3684</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>0.0697/ 1509</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>0.0955/ 2068</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>0.0936/ 2025</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>0.0395/ 856</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>21646</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>0.5315/ 11504</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>0.1702/ 3684</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>0.0697/ 1509</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>0.0955/ 2068</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>0.0936/ 2025</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>0.0395/ 856</t>
         </is>
       </c>
     </row>
@@ -968,7 +1178,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G15"/>
+  <dimension ref="A1:G21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1493,6 +1703,216 @@
       <c r="G15" t="inlineStr">
         <is>
           <t>0.011/ 181</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>16398</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>0.2578/ 4228</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>0.1817/ 2979</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>0.1127/ 1848</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>0.1701/ 2789</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>0.2476/ 4060</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>0.0301/ 494</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>16398</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>0.1356/ 2223</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>0.1165/ 1910</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>0.0957/ 1570</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>0.2098/ 3441</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>0.308/ 5051</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>0.1343/ 2203</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>16398</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>0.3421/ 5610</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>0.2283/ 3744</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>0.1347/ 2209</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>0.1842/ 3020</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>0.0998/ 1636</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>0.0109/ 179</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>16398</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>0.1738/ 2850</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>0.1517/ 2487</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>0.1139/ 1868</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>0.2327/ 3815</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>0.2159/ 3540</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>0.1121/ 1838</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>16398</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>0.1364/ 2237</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>0.1196/ 1961</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>0.0961/ 1576</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>0.2117/ 3472</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>0.3037/ 4980</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>0.1325/ 2172</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>16398</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>0.176/ 2886</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>0.1531/ 2511</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>0.1112/ 1824</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>0.232/ 3805</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>0.2156/ 3536</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>0.112/ 1836</t>
         </is>
       </c>
     </row>
@@ -1507,7 +1927,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H15"/>
+  <dimension ref="A1:H21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2110,6 +2530,246 @@
         </is>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>189241</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>0.042/ 7944</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>0.0398/ 7528</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>0.0384/ 7264</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>0.1012/ 19153</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>0.1621/ 30680</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>0.3087/ 58426</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>0.3078/ 58246</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>189241</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>0.0276/ 5229</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>0.0282/ 5343</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>0.0274/ 5193</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>0.0773/ 14634</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>0.1401/ 26516</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>0.2911/ 55091</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>0.4081/ 77235</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>189241</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>0.093/ 17595</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>0.0904/ 17099</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>0.0874/ 16532</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>0.2202/ 41672</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>0.2603/ 49261</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>0.2217/ 41960</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>0.0271/ 5122</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>189241</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>0.0526/ 9946</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>0.0511/ 9666</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>0.0495/ 9371</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>0.1342/ 25399</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>0.2014/ 38109</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>0.2829/ 53530</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>0.2284/ 43220</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>189241</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>0.0275/ 5210</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>0.0285/ 5389</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>0.0281/ 5318</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>0.0773/ 14637</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>0.1394/ 26386</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>0.294/ 55642</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>0.4051/ 76659</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>189241</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>0.0513/ 9711</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>0.0512/ 9693</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>0.0492/ 9303</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>0.1332/ 25206</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>0.1994/ 37728</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>0.2859/ 54108</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>0.2298/ 43492</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>